<commit_message>
SNU: record Spring English-course evidence
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_4_To_check.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_4_To_check.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. Spring 2027 (1st semester) list not yet checked.</t>
+          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. SPRING evidence (UCEAP / UT Austin exchange records + LikeSNU last-offered semester): 208.228A Geography of Population Change and Migration (English, last offered Spring 2025) and 208.321 Field Study in Geography (English, last offered Spring 2025) - at most 2 English geography courses in Spring; other Spring 2026 geography courses (208.207 Urban Geography, 208.219 Intro Physical Geography, 208.328 Environmental Hazards and Society) have no evidence of English teaching. Not enough English Geography provision in either semester without SNU confirmation.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. Spring 2027 (1st semester) list not yet checked.</t>
+          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. SPRING evidence (UCEAP / UT Austin exchange records + LikeSNU last-offered semester): 208.228A Geography of Population Change and Migration (English, last offered Spring 2025) and 208.321 Field Study in Geography (English, last offered Spring 2025) - at most 2 English geography courses in Spring; other Spring 2026 geography courses (208.207 Urban Geography, 208.219 Intro Physical Geography, 208.328 Environmental Hazards and Society) have no evidence of English teaching. Not enough English Geography provision in either semester without SNU confirmation.</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Remove Seoul National University (insufficient English-taught Geography)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/CurriculumMapping_Geo_4_To_check.xlsx
+++ b/curriculum_mapping_2026-27/CurriculumMapping_Geo_4_To_check.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Rows removed (not usable)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Geography BA'!$A$1:$K$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Geography BSc'!$A$1:$K$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Rows removed (not usable)'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,12 +67,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9F2D0"/>
+        <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00D9F2D0"/>
       </patternFill>
     </fill>
     <fill>
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -555,7 +555,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Seoul National University</t>
+          <t>University of Groningen</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -564,35 +564,35 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. SPRING evidence (UCEAP / UT Austin exchange records + LikeSNU last-offered semester): 208.228A Geography of Population Change and Migration (English, last offered Spring 2025) and 208.321 Field Study in Geography (English, last offered Spring 2025) - at most 2 English geography courses in Spring; other Spring 2026 geography courses (208.207 Urban Geography, 208.219 Intro Physical Geography, 208.328 Environmental Hazards and Society) have no evidence of English teaching. Not enough English Geography provision in either semester without SNU confirmation.</t>
+          <t>Faculty access: confirmed list says UoL students apply to Faculty of Arts / Science and Engineering, but most usable modules are Faculty of Spatial Sciences (FSS does run an exchange course, GESPSP2). Confirm with Study Abroad. Also the workbook's original Groningen rows are Semester 1 (wrong term).</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Spring Semester 1 (Mar-Jun - UoL Semester 2) OR Fall Semester 2 (Sep-Dec - UoL Semester 1)</t>
+          <t>Semester 2</t>
         </is>
       </c>
       <c r="H5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="I5" s="3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Seoul National University</t>
+          <t>University of Groningen</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -601,35 +601,35 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester) checked from the SNU course list: the Geography Department offers only ONE English-taught undergraduate course (208.407A The Politics of Space and Geopolitics); all other geography courses, including the handbook ones (208.302 Geography of Korea, 208.421A History of Geographical Space and Thoughts, 205.242A Population Change and Aging Society), are taught in Korean. 2 English-taught usable modules found, 4 needed -&gt; NOT enough for Fall 2026. SPRING evidence (UCEAP / UT Austin exchange records + LikeSNU last-offered semester): 208.228A Geography of Population Change and Migration (English, last offered Spring 2025) and 208.321 Field Study in Geography (English, last offered Spring 2025) - at most 2 English geography courses in Spring; other Spring 2026 geography courses (208.207 Urban Geography, 208.219 Intro Physical Geography, 208.328 Environmental Hazards and Society) have no evidence of English teaching. Not enough English Geography provision in either semester without SNU confirmation.</t>
+          <t>Faculty access: confirmed list says UoL students apply to Faculty of Arts / Science and Engineering, but most usable modules are Faculty of Spatial Sciences (FSS does run an exchange course, GESPSP2). Confirm with Study Abroad. Also the workbook's original Groningen rows are Semester 1 (wrong term).</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Spring Semester 1 (Mar-Jun - UoL Semester 2) OR Fall Semester 2 (Sep-Dec - UoL Semester 1)</t>
+          <t>Semester 2</t>
         </is>
       </c>
       <c r="H6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>University of Groningen</t>
+          <t>Vrije Universiteit Amsterdam</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -638,17 +638,17 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Faculty access: confirmed list says UoL students apply to Faculty of Arts / Science and Engineering, but most usable modules are Faculty of Spatial Sciences (FSS does run an exchange course, GESPSP2). Confirm with Study Abroad. Also the workbook's original Groningen rows are Semester 1 (wrong term).</t>
+          <t>6 English-taught modules in Semester 2 (P4-P6), 5 needed (30 EC). AB_1318 and AB_1271 removed: taught in Dutch (all other rows checked: English). Minimum met. Confirm exchange access with VU International Office.</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="H7" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>2</v>
@@ -666,7 +666,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>University of Groningen</t>
+          <t>Vrije Universiteit Amsterdam</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -675,17 +675,17 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Faculty access: confirmed list says UoL students apply to Faculty of Arts / Science and Engineering, but most usable modules are Faculty of Spatial Sciences (FSS does run an exchange course, GESPSP2). Confirm with Study Abroad. Also the workbook's original Groningen rows are Semester 1 (wrong term).</t>
+          <t>4 English-taught modules in Semester 2 (P4-P6), 5 needed (30 EC). AB_1318 and AB_1271 removed: taught in Dutch (all other rows checked: English). NOT enough - short by 1. Confirm exchange access with VU International Office.</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -694,83 +694,9 @@
         </is>
       </c>
       <c r="H8" s="3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>6 English-taught modules in Semester 2 (P4-P6), 5 needed (30 EC). AB_1318 and AB_1271 removed: taught in Dutch (all other rows checked: English). Minimum met. Confirm exchange access with VU International Office.</t>
-        </is>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Semester 2</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="I9" s="3" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>4 English-taught modules in Semester 2 (P4-P6), 5 needed (30 EC). AB_1318 and AB_1271 removed: taught in Dutch (all other rows checked: English). NOT enough - short by 1. Confirm exchange access with VU International Office.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Semester 2</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I10" s="3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -785,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -861,7 +787,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Seoul National University — South Korea</t>
+          <t>University of Groningen — Netherlands</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -871,7 +797,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -881,12 +807,12 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>208.407A The Politics of Space and Geopolitics (3 credits)</t>
+          <t>GEEP Environment and Planning (5 ECTS)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -896,25 +822,25 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester, Sep-Dec) - English-taught</t>
+          <t>Semester 2b 2026-27</t>
         </is>
       </c>
       <c r="I2" s="5" t="n"/>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Host: https://sugang.snu.ac.kr/ (SNU Course Search export, 2026 2nd semester (Fall, Sep-Dec 2026), English-taught - provided Oct 2026) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEP | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Seoul National University — South Korea</t>
+          <t>University of Groningen — Netherlands</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -924,7 +850,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+          <t>SOES277 GIS FOR SOCIAL SCIENCES</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -934,12 +860,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>5271.321 Park and Open Space Planning (3 credits)</t>
+          <t>GEGIS Geographic Information Systems (10 ECTS)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -949,290 +875,290 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester, Sep-Dec) - English-taught</t>
+          <t>Semester 2b 2026-27</t>
         </is>
       </c>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Host: https://sugang.snu.ac.kr/ (SNU Course Search export, 2026 2nd semester (Fall, Sep-Dec 2026), English-taught - provided Oct 2026) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGIS | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>University of Groningen — Netherlands</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>GEEP Environment and Planning (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>GEGPLEU Geography, Planning and European Union (5 ECTS)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2a 2026-27</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGPLEU | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>GEPOPGEO Population Geographies (10 ECTS)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2a 2026-27</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEPOPGEO | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>SOES220 CITIES AND REGIONS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>GERG Rural Geography (5 ECTS)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Semester 2b 2026-27</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEP | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GERG | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>University of Groningen — Netherlands</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>SOES277 GIS FOR SOCIAL SCIENCES</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>GEGIS Geographic Information Systems (10 ECTS)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>GESPSP2 Spatial Problems and Spatial Policies: The Dutch Experience (10 ECTS)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Bachelor</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2 2026-27 (exchange course)</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GESPSP2 | NEW (catalogue search to fill gap, Oct 2026) | Course designed for FSS exchange students | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Course designed for FSS exchange students</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>UCG3HU08 The City (5 ECTS)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Semester 2b 2026-27</t>
         </is>
       </c>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGIS | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>GEGPLEU Geography, Planning and European Union (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2a 2026-27</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGPLEU | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>GEPOPGEO Population Geographies (10 ECTS)</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2a 2026-27</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEPOPGEO | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>SOES220 CITIES AND REGIONS</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>GERG Rural Geography (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2b 2026-27</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GERG | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/UCG3HU08 | NEW (catalogue search to fill gap, Oct 2026) | University College Groningen - check exchange access | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; University College Groningen - check exchange access</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>University of Groningen — Netherlands</t>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1242,7 +1168,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>SOES222 PLANNING FOR SUSTAINABLE URBANISM</t>
+          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -1252,12 +1178,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>GESPSP2 Spatial Problems and Spatial Policies: The Dutch Experience (10 ECTS)</t>
+          <t>E_EBE2_ETE Environmental and Transport Economics (6 EC)</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Bachelor</t>
+          <t>Level 3</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1267,71 +1193,71 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Semester 2 2026-27 (exchange course)</t>
+          <t>Period 5 (Semester 2) 2026-27; taught in English</t>
         </is>
       </c>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GESPSP2 | NEW (catalogue search to fill gap, Oct 2026) | Course designed for FSS exchange students | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/E_EBE2_ETE | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
         <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Course designed for FSS exchange students</t>
+          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>UCG3HU08 The City (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2b 2026-27</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/UCG3HU08 | NEW (catalogue search to fill gap, Oct 2026) | University College Groningen - check exchange access | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; University College Groningen - check exchange access</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>E_EBE3_IGS Inclusive Growth and Sustainability (6 EC)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/E_EBE3_IGS | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
@@ -1348,7 +1274,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
+          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -1358,12 +1284,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>E_EBE2_ETE Environmental and Transport Economics (6 EC)</t>
+          <t>L_AABACIW206 Globalisation and Localisation (6 EC)</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 2</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
@@ -1373,69 +1299,69 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Period 5 (Semester 2) 2026-27; taught in English</t>
+          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
         </is>
       </c>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/E_EBE2_ETE | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABACIW206 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Vrije Universiteit Amsterdam — Netherlands</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Geography BA</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>SOES224 POLITICAL ECONOMIES OF CRISIS AND CHANGE</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>E_EBE3_IGS Inclusive Growth and Sustainability (6 EC)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>L_AABAMKD207 Urban Culture and Public Space (6 EC)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>Period 5 (Semester 2) 2026-27; exchange course</t>
         </is>
       </c>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/E_EBE3_IGS | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABAMKD207 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
         </is>
@@ -1454,7 +1380,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>SOES275 SOCIAL AND CULTURAL GEOGRAPHIES</t>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
@@ -1464,7 +1390,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>L_AABACIW206 Globalisation and Localisation (6 EC)</t>
+          <t>L_AABAMKD222 Mediating Environments (6 EC)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1479,182 +1405,76 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
+          <t>Period 4 (Semester 2) 2026-27; taught in English</t>
         </is>
       </c>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="inlineStr">
         <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABACIW206 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABAMKD222 | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
+          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Geography BA</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>S_HDSD The Human Dimension of Sustainable Development: From Ideal to Reality (6 EC)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/S_HDSD | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
           <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>SOES225 THEMES IN URBAN GEOGRAPHY</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>L_AABAMKD207 Urban Culture and Public Space (6 EC)</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="n"/>
-      <c r="J14" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABAMKD207 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K14" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>L_AABAMKD222 Mediating Environments (6 EC)</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Period 4 (Semester 2) 2026-27; taught in English</t>
-        </is>
-      </c>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/L_AABAMKD222 | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Geography BA</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>SOES270 RETHINKING NATURE: ENVIRONMENTAL KNOWLEDGE, SCIENCE AND SOCIETY</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>S_HDSD The Human Dimension of Sustainable Development: From Ideal to Reality (6 EC)</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>Period 5 (Semester 2) 2026-27; exchange course</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="n"/>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/S_HDSD | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K16"/>
+  <autoFilter ref="A1:K14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1665,7 +1485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1741,7 +1561,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Seoul National University — South Korea</t>
+          <t>University of Groningen — Netherlands</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1761,12 +1581,12 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>3345.312 Geochemistry and Lab. (3 credits)</t>
+          <t>GEEE Environment and Engineering (5 ECTS)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -1776,25 +1596,25 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester, Sep-Dec) - English-taught</t>
+          <t>Semester 2a 2026-27</t>
         </is>
       </c>
       <c r="I2" s="5" t="n"/>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Host: https://sugang.snu.ac.kr/ (SNU Course Search export, 2026 2nd semester (Fall, Sep-Dec 2026), English-taught - provided Oct 2026) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEE | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
         <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Seoul National University — South Korea</t>
+          <t>University of Groningen — Netherlands</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -1814,12 +1634,12 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>457.210A Environmental Engineering (section 002, English) (3 credits)</t>
+          <t>GEEP Environment and Planning (5 ECTS)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Level 2</t>
+          <t>Bachelor</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -1829,553 +1649,447 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Fall 2026 (SNU 2nd semester, Sep-Dec) - English-taught</t>
+          <t>Semester 2b 2026-27</t>
         </is>
       </c>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>Host: https://sugang.snu.ac.kr/ (SNU Course Search export, 2026 2nd semester (Fall, Sep-Dec 2026), English-taught - provided Oct 2026) | NEW (Oct 2026 deep check: module confirmed in the 2026/27 timetable for the exchange period) | UoL match is a SUGGESTION for department review</t>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEP | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>Added Oct 2026 (deep check): verified in 2026/27 timetable; UoL match is a suggestion for review</t>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>University of Groningen — Netherlands</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>GEGIS Geographic Information Systems (10 ECTS)</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2b 2026-27</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGIS | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>GELSC Landscapes (5 ECTS)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2b 2026-27</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GELSC | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>GEPG Physical Geography (5 ECTS)</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2a 2026-27</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEPG | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>University of Groningen — Netherlands</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>WBBIP02-06 Artificial Intelligence for Forest and Landscape Remote Sensing (6 ECTS)</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Semester 2a 2026-27</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://ocasys.rug.nl/current/catalog/course/WBBIP02-06 | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Science and Engineering | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Science and Engineering</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>AB_1201 Statistics and Methodology (6 EC)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>Period 4 (Semester 2) 2026-27; exchange course</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1201 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>AB_1288 Big Data in Sustainability Science (6 EC)</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Level 3</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Period 4 (Semester 2) 2026-27</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1288 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Bachelor course not flagged as exchange course - confirm access</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Geography BSc</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>GEEE Environment and Engineering (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2a 2026-27</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEE | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>AB_1357 Planetary Health: PHIACW (6 EC)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>Period 5 (Semester 2) 2026-27</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1357 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Bachelor course not flagged as exchange course - confirm access</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Vrije Universiteit Amsterdam — Netherlands</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Geography BSc</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>SOES214 CHANGING ENVIRONMENTS</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>GEEP Environment and Planning (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2b 2026-27</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEEP | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>GEGIS Geographic Information Systems (10 ECTS)</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2b 2026-27</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEGIS | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>GELSC Landscapes (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2b 2026-27</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GELSC | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K7" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>SOES218 GEOMORPHOLOGY: PROCESSES AND FORMS</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>GEPG Physical Geography (5 ECTS)</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2a 2026-27</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/GEPG | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K8" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Spatial Sciences - confirmed list says UoL students apply to Arts / Science and Engineering; FSS takes exchange students (see GESPSP2) - confirm with Study Abroad</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>University of Groningen — Netherlands</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>SOES269 GIS FOR THE NATURAL ENVIRONMENT</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>WBBIP02-06 Artificial Intelligence for Forest and Landscape Remote Sensing (6 ECTS)</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Bachelor</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>Semester 2a 2026-27</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="n"/>
-      <c r="J9" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://ocasys.rug.nl/current/catalog/course/WBBIP02-06 | NEW (catalogue search to fill gap, Oct 2026) | Faculty of Science and Engineering | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K9" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Faculty of Science and Engineering</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>AB_1201 Statistics and Methodology (6 EC)</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Period 4 (Semester 2) 2026-27; exchange course</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1201 | NEW (catalogue search to fill gap, Oct 2026) | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K10" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>AB_1288 Big Data in Sustainability Science (6 EC)</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Level 3</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>Period 4 (Semester 2) 2026-27</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n"/>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1288 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Level 5</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>AB_470074 Urban Ecology (6 EC)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Level 2</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Period 6 (Semester 2) 2026-27</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_470074 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Bachelor course not flagged as exchange course - confirm access</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>AB_1357 Planetary Health: PHIACW (6 EC)</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>Period 5 (Semester 2) 2026-27</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_1357 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K12" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Bachelor course not flagged as exchange course - confirm access</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Vrije Universiteit Amsterdam — Netherlands</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Geography BSc</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>SOES214 CHANGING ENVIRONMENTS</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Level 5</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>AB_470074 Urban Ecology (6 EC)</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>Level 2</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Period 6 (Semester 2) 2026-27</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="n"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Host: https://studiegids.vu.nl/en/courses/2026-2027/AB_470074 | NEW (catalogue search to fill gap, Oct 2026) | Bachelor course not flagged as exchange course - confirm access | UoL match is a SUGGESTION for department review</t>
-        </is>
-      </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>Added Oct 2026: catalogue search to fill gap; UoL match is a suggestion for review; Bachelor course not flagged as exchange course - confirm access</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K13"/>
+  <autoFilter ref="A1:K11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>